<commit_message>
Resolve conflicts, update protocol files, and optimize anchor calibration solver
</commit_message>
<xml_diff>
--- a/reference/uwb_calibration.xlsx
+++ b/reference/uwb_calibration.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\uwb-rtls\reference\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\final_project\uwb-rtls\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D56B3F8D-3A31-4EFF-A02F-4227BF78A2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E231B86E-EBE6-4DB7-9D29-597C82430D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{43766B12-A4F5-4323-B206-359946D7DF34}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Antenna Delay</t>
   </si>
@@ -44,14 +44,26 @@
     <t>Anchor</t>
   </si>
   <si>
-    <t>Distance</t>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>(0,0)</t>
+  </si>
+  <si>
+    <t>(0,976)</t>
+  </si>
+  <si>
+    <t>(976,0)</t>
+  </si>
+  <si>
+    <t>(976,976)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -59,31 +71,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -100,9 +107,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,10 +444,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D738D6E6-D2D2-48FE-AA05-6713A3561588}">
-  <dimension ref="A4:E10"/>
+  <dimension ref="A4:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -451,86 +458,61 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>732</v>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="1">
-        <v>16688</v>
-      </c>
-      <c r="D5" s="3">
-        <v>16588</v>
-      </c>
-      <c r="E5">
-        <v>16611</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="3">
+        <v>16439</v>
+      </c>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
       <c r="B6">
         <v>2</v>
       </c>
-      <c r="D6" s="2">
-        <v>16562</v>
-      </c>
-      <c r="E6">
-        <v>16611</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>732</v>
+      <c r="C6" s="3">
+        <v>16440</v>
+      </c>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
       </c>
       <c r="B7">
         <v>3</v>
       </c>
-      <c r="C7" s="1">
-        <v>16605</v>
-      </c>
-      <c r="D7" s="3">
-        <v>16618</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>976</v>
+      <c r="C7" s="3">
+        <v>16435</v>
+      </c>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="B8">
         <v>4</v>
       </c>
-      <c r="C8" s="1">
-        <v>16630</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>488</v>
-      </c>
-      <c r="B9">
-        <v>4</v>
-      </c>
-      <c r="C9" s="1">
-        <v>16568</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>732</v>
-      </c>
-      <c r="B10">
-        <v>4</v>
-      </c>
-      <c r="C10" s="1">
-        <v>16655</v>
-      </c>
-      <c r="D10" s="3">
-        <v>16593</v>
-      </c>
-      <c r="E10">
-        <v>16681</v>
-      </c>
+      <c r="C8" s="3">
+        <v>16437</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
(exxcel) save antenna delay
</commit_message>
<xml_diff>
--- a/reference/uwb_calibration.xlsx
+++ b/reference/uwb_calibration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\final_project\uwb-rtls\reference\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HOC\S\STM32\IDE\DATN\uwb-rtls\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E231B86E-EBE6-4DB7-9D29-597C82430D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{255ACB1B-0BAB-4521-B930-518FB197A41F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{43766B12-A4F5-4323-B206-359946D7DF34}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{43766B12-A4F5-4323-B206-359946D7DF34}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -108,8 +108,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -444,10 +444,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D738D6E6-D2D2-48FE-AA05-6713A3561588}">
-  <dimension ref="A4:D10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A4:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -458,7 +462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -468,9 +472,14 @@
       <c r="C5" s="3">
         <v>16439</v>
       </c>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D5" s="3">
+        <v>16436</v>
+      </c>
+      <c r="E5">
+        <v>16318</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -480,9 +489,14 @@
       <c r="C6" s="3">
         <v>16440</v>
       </c>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D6" s="3">
+        <v>16361</v>
+      </c>
+      <c r="E6">
+        <v>16361</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -492,9 +506,14 @@
       <c r="C7" s="3">
         <v>16435</v>
       </c>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D7" s="3">
+        <v>16329</v>
+      </c>
+      <c r="E7">
+        <v>16278</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -504,13 +523,18 @@
       <c r="C8" s="3">
         <v>16437</v>
       </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D8" s="3">
+        <v>16234</v>
+      </c>
+      <c r="E8">
+        <v>16283</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
     </row>

</xml_diff>